<commit_message>
data for synthetic companies added
</commit_message>
<xml_diff>
--- a/data/semi_structured/Investment_AI_Analyst_Estimates_Q2_2026.xlsx
+++ b/data/semi_structured/Investment_AI_Analyst_Estimates_Q2_2026.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Estimates" sheetId="1" r:id="R19db9085522a4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Estimates" sheetId="1" r:id="Rea7457bde7334c2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48,7 +48,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -85,6 +85,7 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -302,8 +303,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
@@ -313,7 +314,7 @@
   <x:sheetData>
     <x:row r="1" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A1" s="10" t="str">
-        <x:v>Ticker</x:v>
+        <x:v>Security ID</x:v>
       </x:c>
       <x:c r="B1" s="10" t="str">
         <x:v>Company</x:v>
@@ -336,10 +337,10 @@
     </x:row>
     <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>NOVA</x:v>
+        <x:v>IA-SYN-01</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>NovaChip Technologies</x:v>
+        <x:v>Synthetic Compute Company 01</x:v>
       </x:c>
       <x:c r="C2" s="14" t="n">
         <x:v>1.25</x:v>
@@ -359,10 +360,10 @@
     </x:row>
     <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A3" s="11" t="str">
-        <x:v>EVRG</x:v>
+        <x:v>IA-SYN-02</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
-        <x:v>Evergreen Energy Systems</x:v>
+        <x:v>Synthetic Energy Company 02</x:v>
       </x:c>
       <x:c r="C3" s="14" t="n">
         <x:v>2.1</x:v>
@@ -382,10 +383,10 @@
     </x:row>
     <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
-        <x:v>APXR</x:v>
+        <x:v>IA-SYN-03</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>Apex Retail Group</x:v>
+        <x:v>Synthetic Retail Company 03</x:v>
       </x:c>
       <x:c r="C4" s="14" t="n">
         <x:v>3.4</x:v>
@@ -405,10 +406,10 @@
     </x:row>
     <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="11" t="str">
-        <x:v>MDHN</x:v>
+        <x:v>IA-SYN-04</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Meridian Health Systems</x:v>
+        <x:v>Synthetic Health Company 04</x:v>
       </x:c>
       <x:c r="C5" s="14" t="n">
         <x:v>2.85</x:v>
@@ -428,10 +429,10 @@
     </x:row>
     <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A6" s="11" t="str">
-        <x:v>VTXI</x:v>
+        <x:v>IA-SYN-05</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>Vertex Industrial Technologies</x:v>
+        <x:v>Synthetic Industrial Company 05</x:v>
       </x:c>
       <x:c r="C6" s="14" t="n">
         <x:v>1.72</x:v>
@@ -452,7 +453,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb90da75ac6d64ece"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fad067c73ed4165"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>